<commit_message>
Update configurator API endpoint and data with image URLs
New Apps Script deployment pointing to fresh Google Sheet.
Updated XLSX includes Webflow CDN image URLs for G9 exteriors,
interiors, wheels, and accessories.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/configurator-data/xpeng-configurator-data.xlsx
+++ b/configurator-data/xpeng-configurator-data.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,23 +30,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8E8E8"/>
-        <bgColor rgb="00E8E8E8"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -61,9 +51,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,30 +420,24 @@
   </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>model_slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>model_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>starting_price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>hero_image</t>
         </is>
@@ -521,126 +504,104 @@
   </sheetPr>
   <dimension ref="A1:T10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>model_slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>variant_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>variant_name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>is_default</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>range_km</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>power_kw</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>torque_nm</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>acceleration</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>top_speed</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>battery_kwh</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>battery_type</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>dc_charge_power_kw</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>dc_charge_time</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ac_charge_time</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>energy_consumption</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>drivetrain</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>suspension</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>delivery_time</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -1415,72 +1376,59 @@
   </sheetPr>
   <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>model_slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>variant_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>color_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>color_name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>color_hex</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>is_default</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>image_front</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>image_side</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>image_rear</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -1518,7 +1466,11 @@
       <c r="G2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6841d529bf62df8e50_g9-arctic-white-side.webp</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
@@ -1557,7 +1509,11 @@
       <c r="G3" t="b">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6841d529bf62df8e6a_g9-silver-frost-side.webp</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
@@ -1596,7 +1552,11 @@
       <c r="G4" t="b">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d691a61eba809ab6e41_g9-midnight-black-side.webp</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
@@ -1616,12 +1576,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>matte-gray</t>
+          <t>graphite-gray</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Matte Gray</t>
+          <t>Graphite Gray</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1635,7 +1595,11 @@
       <c r="G5" t="b">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6905a55be18cfe5df5_g9-graphite-gray-side.webp</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
@@ -2006,60 +1970,49 @@
   </sheetPr>
   <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>model_slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>variant_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>interior_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>interior_name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>is_default</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>image_thumb</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>image_full</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -2092,7 +2045,11 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d69f40b6da4eafccb4d_g9-interior-black.webp</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>1</v>
@@ -2125,7 +2082,11 @@
       <c r="F3" t="b">
         <v>0</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6a4ff40eddce423e22_g9-interior-coffee.webp</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>2</v>
@@ -2375,54 +2336,44 @@
   </sheetPr>
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>model_slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>variant_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>wheel_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>wheel_name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>is_default</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>image_thumb</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -2455,7 +2406,11 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6ac972d2b0ba331f5e_g9-wheel-20.webp</t>
+        </is>
+      </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
@@ -2729,54 +2684,44 @@
   </sheetPr>
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>model_slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>variant_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>accessory_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>accessory_name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>image</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -2811,7 +2756,11 @@
           <t>Electrically retractable tow hitch with max towing capacity 1500 kg (braked) / 750 kg (unbraked).</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6a4ff40eddce423e56_g9-tow-bar.webp</t>
+        </is>
+      </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Make configurator options panel scrollable
Add overflow-y auto + max-height 100vh to options panel.
Update XLSX with corrected prices, 4 interiors, 2 wheels,
premium package matching German configurator.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/configurator-data/xpeng-configurator-data.xlsx
+++ b/configurator-data/xpeng-configurator-data.xlsx
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>71600</v>
+        <v>72600</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -1533,17 +1533,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>midnight-black</t>
+          <t>graphite-gray</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Midnight Black</t>
+          <t>Graphite Gray</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>#2D2D2D</t>
+          <t>#707070</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d691a61eba809ab6e41_g9-midnight-black-side.webp</t>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6905a55be18cfe5df5_g9-graphite-gray-side.webp</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -1576,28 +1576,28 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>graphite-gray</t>
+          <t>midnight-black</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Graphite Gray</t>
+          <t>Midnight Black</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>#707070</t>
+          <t>#2D2D2D</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6905a55be18cfe5df5_g9-graphite-gray-side.webp</t>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d691a61eba809ab6e41_g9-midnight-black-side.webp</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -1968,7 +1968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2031,12 +2031,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>meteorite-black</t>
+          <t>black-leatherette</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Meteorite Black</t>
+          <t>Black Leatherette</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>coffee-brown</t>
+          <t>coffee-leatherette</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Coffee Brown</t>
+          <t>Coffee Leatherette</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -2095,7 +2095,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>g6</t>
+          <t>g9</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2105,30 +2105,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>black-leatherette</t>
+          <t>saddle-leatherette</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Black Leatherette</t>
+          <t>Saddle Leatherette</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a156f092372a37540341f5b_g9-interior-saddle.webp</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>g6</t>
+          <t>g9</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2152,31 +2156,35 @@
       <c r="F5" t="b">
         <v>0</v>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a156f0911a8e6ceceeac25b_g9-interior-gray.webp</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>p7-plus</t>
+          <t>g6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>rwd-sr</t>
+          <t>all</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>black-pu</t>
+          <t>black-leatherette</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Black PU</t>
+          <t>Black Leatherette</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -2194,34 +2202,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>p7-plus</t>
+          <t>g6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>rwd-lr</t>
+          <t>all</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>black-nappa</t>
+          <t>gray-leatherette</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Black Nappa Leather</t>
+          <t>Gray Leatherette</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -2232,29 +2240,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rwd-lr</t>
+          <t>rwd-sr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>white-nappa</t>
+          <t>black-pu</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>White Nappa Leather</t>
+          <t>Black PU</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2265,7 +2273,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>awd</t>
+          <t>rwd-lr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2298,7 +2306,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>awd</t>
+          <t>rwd-lr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2320,6 +2328,72 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>p7-plus</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>awd</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>black-nappa</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Black Nappa Leather</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>p7-plus</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>awd</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>white-nappa</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>White Nappa Leather</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2334,7 +2408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2397,7 +2471,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>20" Standard</t>
+          <t>20" Alloy Wheels</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -2418,33 +2492,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>g6</t>
+          <t>g9</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>rwd-sr</t>
+          <t>all</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>18-aero</t>
+          <t>21-sport</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>18" Aero</t>
+          <t>21" Sport Wheels</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1260</v>
       </c>
       <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a156f096e7ca3d0bc68c88f_g9-wheel-21.webp</t>
+        </is>
+      </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2460,23 +2538,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>20-sport</t>
+          <t>18-aero</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>20" Sport</t>
+          <t>18" Aero</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -2487,28 +2565,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>rwd-lr</t>
+          <t>rwd-sr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>18-aero</t>
+          <t>20-sport</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>18" Aero</t>
+          <t>20" Sport</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -2524,23 +2602,23 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20-sport</t>
+          <t>18-aero</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>20" Sport</t>
+          <t>18" Aero</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -2551,7 +2629,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>awd</t>
+          <t>rwd-lr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2568,32 +2646,32 @@
         <v>0</v>
       </c>
       <c r="F7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>p7-plus</t>
+          <t>g6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rwd-sr</t>
+          <t>awd</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>19-standard</t>
+          <t>20-sport</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>19" Standard</t>
+          <t>20" Sport</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -2615,17 +2693,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>rwd-lr</t>
+          <t>rwd-sr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>20-performance</t>
+          <t>19-standard</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>20" Performance</t>
+          <t>19" Standard</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -2647,7 +2725,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>awd</t>
+          <t>rwd-lr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2668,6 +2746,38 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>p7-plus</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>awd</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>20-performance</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>20" Performance</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2682,7 +2792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2740,25 +2850,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>tow-hitch</t>
+          <t>premium-package</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Electric Retractable Tow Hitch</t>
+          <t>Premium Package</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1260</v>
+        <v>3960</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Electrically retractable tow hitch with max towing capacity 1500 kg (braked) / 750 kg (unbraked).</t>
+          <t>Nappa leather seats, 4-seat massage, rear seat ventilation, suede headliner, enhanced lumbar support, Dynaudio XOPERA sound system.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6a4ff40eddce423e56_g9-tow-bar.webp</t>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a156f09a8ad7b89ea79a21f_g9-premium-package.webp</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -2768,7 +2878,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>g6</t>
+          <t>g9</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2787,22 +2897,26 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1160</v>
+        <v>1260</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Electrically retractable tow hitch with max towing capacity 1500 kg (braked) / 750 kg (unbraked).</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/6a041f81e8910a5a1669594c/6a155d6a4ff40eddce423e56_g9-tow-bar.webp</t>
+        </is>
+      </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>p7-plus</t>
+          <t>g6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2821,7 +2935,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1190</v>
+        <v>1160</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2830,6 +2944,40 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>p7-plus</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>tow-hitch</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Electric Retractable Tow Hitch</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1190</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Electrically retractable tow hitch with max towing capacity 1500 kg (braked) / 750 kg (unbraked).</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>